<commit_message>
Add market config (assets, sessions); journal Sessione/MAE columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8etLe3AX5XxrJJdQQAzeE
</commit_message>
<xml_diff>
--- a/journal/trading_journal.xlsx
+++ b/journal/trading_journal.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,6 +486,16 @@
       <c r="N1" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Sessione</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>MAE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add market structure trend (H4/H1 HH/HL); journal trend columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8etLe3AX5XxrJJdQQAzeE
</commit_message>
<xml_diff>
--- a/journal/trading_journal.xlsx
+++ b/journal/trading_journal.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,6 +496,21 @@
       <c r="P1" t="inlineStr">
         <is>
           <t>MAE</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Trend H4</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Trend H1</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Controtendenza</t>
         </is>
       </c>
     </row>

</xml_diff>